<commit_message>
Restyle Woodbridge chart to match Will's example
Switches the combo chart to the maroon + navy palette used in the
Market vs. Vacancy example (Net Absorption dark maroon, SF Delivered
brick, Market Rent Growth dark navy line), drops the secondary
gridlines, and adds a matplotlib preview script so the look can be
reviewed without opening Excel.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017toQ13hPwjGEJYmbhu47L5
</commit_message>
<xml_diff>
--- a/scratchpad/Woodbridge_Industrial_Chart.xlsx
+++ b/scratchpad/Woodbridge_Industrial_Chart.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="#,##0;[Red](#,##0);&quot;—&quot;"/>
+    <numFmt numFmtId="164" formatCode="#,##0;[Red](#,##0);&quot;-&quot;"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -30,7 +30,7 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001F3864"/>
+      <color rgb="00000000"/>
       <sz val="14"/>
     </font>
     <font>
@@ -196,7 +196,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Woodbridge Industrial — Net Absorption &amp; SF Delivered with Market Rent Growth</a:t>
+              <a:t>Woodbridge - Absorption vs. Deliveries</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -216,9 +216,12 @@
           </tx>
           <spPr>
             <a:solidFill>
-              <a:srgbClr val="4472C4"/>
+              <a:srgbClr val="963634"/>
             </a:solidFill>
             <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="963634"/>
+              </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -243,9 +246,12 @@
           </tx>
           <spPr>
             <a:solidFill>
-              <a:srgbClr val="ED7D31"/>
+              <a:srgbClr val="C0504D"/>
             </a:solidFill>
             <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="C0504D"/>
+              </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -260,7 +266,8 @@
             </numRef>
           </val>
         </ser>
-        <gapWidth val="90"/>
+        <gapWidth val="80"/>
+        <overlap val="-10"/>
         <axId val="10"/>
         <axId val="100"/>
       </barChart>
@@ -277,21 +284,21 @@
           <spPr>
             <a:ln w="28000">
               <a:solidFill>
-                <a:srgbClr val="A5A5A5"/>
+                <a:srgbClr val="1F3864"/>
               </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="circle"/>
-            <size val="7"/>
+            <size val="6"/>
             <spPr>
               <a:solidFill>
-                <a:srgbClr val="A5A5A5"/>
+                <a:srgbClr val="1F3864"/>
               </a:solidFill>
               <a:ln>
                 <a:solidFill>
-                  <a:srgbClr val="A5A5A5"/>
+                  <a:srgbClr val="1F3864"/>
                 </a:solidFill>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -313,21 +320,6 @@
           <orientation val="minMax"/>
         </scaling>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Year</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
@@ -341,7 +333,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln>
+            <a:ln w="6350">
               <a:solidFill>
                 <a:srgbClr val="D9D9D9"/>
               </a:solidFill>
@@ -358,7 +350,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>SF</a:t>
+                  <a:t>Square Feet</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -375,7 +367,6 @@
           <orientation val="minMax"/>
         </scaling>
         <axPos val="l"/>
-        <majorGridlines/>
         <title>
           <tx>
             <rich>
@@ -385,7 +376,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Market Rent Growth (%)</a:t>
+                  <a:t>Market Rent Growth</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -735,14 +726,14 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Woodbridge Industrial Submarket — Net Absorption, Deliveries &amp; Rent Growth</t>
+          <t>Woodbridge - Absorption, Deliveries &amp; Rent Growth</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Annual, 2016–2026  |  Source: CoStar (All Properties → Industrial, ≥20,000 SF)</t>
+          <t>Annual, 2016-2026  |  Source: CoStar (All Properties -&gt; Industrial, &gt;=20,000 SF)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Woodbridge Market vs. Vacancy chart, finishing the set
Rebuilds the Woodbridge workbook as two sheets matching the I-95
Corridor layout: Market Rent ($/SF) bars + Vacancy Rate line on the
first sheet, Net Absorption + SF Delivered twin bars + Market Rent
Growth line on the second. Both capped at 2026 with the maroon/navy
palette. Refreshes the preview renders accordingly.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017toQ13hPwjGEJYmbhu47L5
</commit_message>
<xml_diff>
--- a/scratchpad/Woodbridge_Industrial_Chart.xlsx
+++ b/scratchpad/Woodbridge_Industrial_Chart.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Woodbridge" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Market vs Vacancy" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Absorption vs Deliveries" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,8 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="#,##0;[Red](#,##0);&quot;-&quot;"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="#,##0;[Red](#,##0);&quot;-&quot;"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -89,11 +91,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -105,6 +105,9 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="10" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -196,7 +199,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Woodbridge - Absorption vs. Deliveries</a:t>
+              <a:t>Woodbridge Industrial - Market vs. Vacancy</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -211,7 +214,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Woodbridge'!B4</f>
+              <f>'Market vs Vacancy'!B4</f>
             </strRef>
           </tx>
           <spPr>
@@ -227,58 +230,27 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Woodbridge'!$A$5:$A$15</f>
+              <f>'Market vs Vacancy'!$A$5:$A$15</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Woodbridge'!$B$5:$B$15</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
-              <f>'Woodbridge'!C4</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="C0504D"/>
-            </a:solidFill>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="C0504D"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Woodbridge'!$A$5:$A$15</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Woodbridge'!$C$5:$C$15</f>
+              <f>'Market vs Vacancy'!$B$5:$B$15</f>
             </numRef>
           </val>
         </ser>
         <gapWidth val="80"/>
-        <overlap val="-10"/>
         <axId val="10"/>
         <axId val="100"/>
       </barChart>
       <lineChart>
         <grouping val="standard"/>
         <ser>
-          <idx val="2"/>
-          <order val="2"/>
+          <idx val="1"/>
+          <order val="1"/>
           <tx>
             <strRef>
-              <f>'Woodbridge'!D4</f>
+              <f>'Market vs Vacancy'!C4</f>
             </strRef>
           </tx>
           <spPr>
@@ -306,7 +278,222 @@
           </marker>
           <val>
             <numRef>
-              <f>'Woodbridge'!$D$5:$D$15</f>
+              <f>'Market vs Vacancy'!$C$5:$C$15</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="200"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines>
+          <spPr>
+            <a:ln w="6350">
+              <a:solidFill>
+                <a:srgbClr val="D9D9D9"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+        </majorGridlines>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Market Rent ($/SF)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <numFmt formatCode="&quot;$&quot;#,##0.00" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+      <valAx>
+        <axId val="200"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Vacancy Rate</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <numFmt formatCode="0.0%" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+        <crosses val="max"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="b"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Woodbridge Industrial - Absorption vs. Deliveries</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Absorption vs Deliveries'!B4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="963634"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="963634"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Absorption vs Deliveries'!$A$5:$A$15</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Absorption vs Deliveries'!$B$5:$B$15</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Absorption vs Deliveries'!C4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="C0504D"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="C0504D"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Absorption vs Deliveries'!$A$5:$A$15</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Absorption vs Deliveries'!$C$5:$C$15</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="80"/>
+        <overlap val="-10"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Absorption vs Deliveries'!D4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="28000">
+              <a:solidFill>
+                <a:srgbClr val="1F3864"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="6"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="1F3864"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="1F3864"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <val>
+            <numRef>
+              <f>'Absorption vs Deliveries'!$D$5:$D$15</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -399,6 +586,33 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7920000" cy="3960000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -714,6 +928,182 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Woodbridge Industrial - Market vs. Vacancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Annual 2016-2026  |  CoStar (All Properties -&gt; Industrial, &gt;=20,000 SF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Market Rent ($/SF)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Vacancy Rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n">
+        <v>2016</v>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>0.02204</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n">
+        <v>2017</v>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>10.15</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>0.0452</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="n">
+        <v>2018</v>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>10.74</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>0.05503</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="n">
+        <v>2019</v>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>11.37</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>0.04733</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>2020</v>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>12.11</v>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>0.03426</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>0.02003</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>14.93</v>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>0.02389</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>16.19</v>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>0.01949</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>17.16</v>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>0.03338</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>18.17</v>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>0.03094</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>18.65</v>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>0.04158</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -726,14 +1116,14 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Woodbridge - Absorption, Deliveries &amp; Rent Growth</t>
+          <t>Woodbridge Industrial - Absorption vs. Deliveries</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Annual, 2016-2026  |  Source: CoStar (All Properties -&gt; Industrial, &gt;=20,000 SF)</t>
+          <t>Annual 2016-2026  |  CoStar (All Properties -&gt; Industrial, &gt;=20,000 SF)</t>
         </is>
       </c>
     </row>
@@ -763,10 +1153,10 @@
       <c r="A5" s="4" t="n">
         <v>2016</v>
       </c>
-      <c r="B5" s="5" t="n">
+      <c r="B5" s="7" t="n">
         <v>100437</v>
       </c>
-      <c r="C5" s="5" t="n"/>
+      <c r="C5" s="7" t="n"/>
       <c r="D5" s="6" t="n">
         <v>0.0564</v>
       </c>
@@ -775,10 +1165,10 @@
       <c r="A6" s="4" t="n">
         <v>2017</v>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B6" s="7" t="n">
         <v>-56411</v>
       </c>
-      <c r="C6" s="5" t="n"/>
+      <c r="C6" s="7" t="n"/>
       <c r="D6" s="6" t="n">
         <v>0.0498</v>
       </c>
@@ -787,10 +1177,10 @@
       <c r="A7" s="4" t="n">
         <v>2018</v>
       </c>
-      <c r="B7" s="5" t="n">
+      <c r="B7" s="7" t="n">
         <v>-23948</v>
       </c>
-      <c r="C7" s="5" t="n"/>
+      <c r="C7" s="7" t="n"/>
       <c r="D7" s="6" t="n">
         <v>0.0576</v>
       </c>
@@ -799,10 +1189,10 @@
       <c r="A8" s="4" t="n">
         <v>2019</v>
       </c>
-      <c r="B8" s="5" t="n">
+      <c r="B8" s="7" t="n">
         <v>18759</v>
       </c>
-      <c r="C8" s="5" t="n"/>
+      <c r="C8" s="7" t="n"/>
       <c r="D8" s="6" t="n">
         <v>0.0585</v>
       </c>
@@ -811,10 +1201,10 @@
       <c r="A9" s="4" t="n">
         <v>2020</v>
       </c>
-      <c r="B9" s="5" t="n">
+      <c r="B9" s="7" t="n">
         <v>31836</v>
       </c>
-      <c r="C9" s="5" t="n"/>
+      <c r="C9" s="7" t="n"/>
       <c r="D9" s="6" t="n">
         <v>0.065</v>
       </c>
@@ -823,10 +1213,10 @@
       <c r="A10" s="4" t="n">
         <v>2021</v>
       </c>
-      <c r="B10" s="5" t="n">
+      <c r="B10" s="7" t="n">
         <v>34656</v>
       </c>
-      <c r="C10" s="5" t="n"/>
+      <c r="C10" s="7" t="n"/>
       <c r="D10" s="6" t="n">
         <v>0.1071</v>
       </c>
@@ -835,10 +1225,10 @@
       <c r="A11" s="4" t="n">
         <v>2022</v>
       </c>
-      <c r="B11" s="5" t="n">
+      <c r="B11" s="7" t="n">
         <v>-9390</v>
       </c>
-      <c r="C11" s="5" t="n"/>
+      <c r="C11" s="7" t="n"/>
       <c r="D11" s="6" t="n">
         <v>0.114</v>
       </c>
@@ -847,10 +1237,10 @@
       <c r="A12" s="4" t="n">
         <v>2023</v>
       </c>
-      <c r="B12" s="5" t="n">
+      <c r="B12" s="7" t="n">
         <v>231444</v>
       </c>
-      <c r="C12" s="5" t="n">
+      <c r="C12" s="7" t="n">
         <v>225124</v>
       </c>
       <c r="D12" s="6" t="n">
@@ -861,10 +1251,10 @@
       <c r="A13" s="4" t="n">
         <v>2024</v>
       </c>
-      <c r="B13" s="5" t="n">
+      <c r="B13" s="7" t="n">
         <v>-36955</v>
       </c>
-      <c r="C13" s="5" t="n"/>
+      <c r="C13" s="7" t="n"/>
       <c r="D13" s="6" t="n">
         <v>0.0603</v>
       </c>
@@ -873,10 +1263,10 @@
       <c r="A14" s="4" t="n">
         <v>2025</v>
       </c>
-      <c r="B14" s="5" t="n">
+      <c r="B14" s="7" t="n">
         <v>114004</v>
       </c>
-      <c r="C14" s="5" t="n">
+      <c r="C14" s="7" t="n">
         <v>110935</v>
       </c>
       <c r="D14" s="6" t="n">
@@ -887,10 +1277,10 @@
       <c r="A15" s="4" t="n">
         <v>2026</v>
       </c>
-      <c r="B15" s="5" t="n">
+      <c r="B15" s="7" t="n">
         <v>-29494</v>
       </c>
-      <c r="C15" s="5" t="n"/>
+      <c r="C15" s="7" t="n"/>
       <c r="D15" s="6" t="n">
         <v>0.0591</v>
       </c>

</xml_diff>